<commit_message>
data: move legacy burst zone marker to spell keyword metadata
</commit_message>
<xml_diff>
--- a/cards.xlsx
+++ b/cards.xlsx
@@ -67251,7 +67251,7 @@
         <v>4786</v>
       </c>
       <c r="R48" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S48" s="5" t="s">
         <v>4787</v>
@@ -67319,7 +67319,7 @@
         <v>4794</v>
       </c>
       <c r="R49" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S49" s="5" t="s">
         <v>4795</v>
@@ -67387,7 +67387,7 @@
         <v>96</v>
       </c>
       <c r="R50" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S50" s="5" t="s">
         <v>4801</v>
@@ -67455,7 +67455,7 @@
         <v>930</v>
       </c>
       <c r="R51" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S51" s="5" t="s">
         <v>4808</v>
@@ -67523,7 +67523,7 @@
         <v>4814</v>
       </c>
       <c r="R52" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S52" s="5" t="s">
         <v>4815</v>
@@ -67591,7 +67591,7 @@
         <v>4821</v>
       </c>
       <c r="R53" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S53" s="5" t="s">
         <v>4822</v>
@@ -67659,7 +67659,7 @@
         <v>4829</v>
       </c>
       <c r="R54" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S54" s="5" t="s">
         <v>4494</v>
@@ -67727,7 +67727,7 @@
         <v>96</v>
       </c>
       <c r="R55" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S55" s="5" t="s">
         <v>4835</v>
@@ -71195,7 +71195,7 @@
         <v>5123</v>
       </c>
       <c r="R106" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S106" s="5" t="s">
         <v>5124</v>
@@ -71263,7 +71263,7 @@
         <v>5130</v>
       </c>
       <c r="R107" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S107" s="5" t="s">
         <v>191</v>
@@ -71331,7 +71331,7 @@
         <v>96</v>
       </c>
       <c r="R108" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S108" s="5" t="s">
         <v>5136</v>
@@ -71399,7 +71399,7 @@
         <v>323</v>
       </c>
       <c r="R109" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S109" s="5" t="s">
         <v>5143</v>
@@ -71467,7 +71467,7 @@
         <v>2584</v>
       </c>
       <c r="R110" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S110" s="5" t="s">
         <v>5149</v>
@@ -71535,7 +71535,7 @@
         <v>472</v>
       </c>
       <c r="R111" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S111" s="5" t="s">
         <v>5155</v>
@@ -71603,7 +71603,7 @@
         <v>5162</v>
       </c>
       <c r="R112" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S112" s="5" t="s">
         <v>5163</v>
@@ -71671,7 +71671,7 @@
         <v>483</v>
       </c>
       <c r="R113" s="5" t="s">
-        <v>2275</v>
+        <v>34</v>
       </c>
       <c r="S113" s="5" t="s">
         <v>5169</v>

</xml_diff>